<commit_message>
Update DSA Question sheet
</commit_message>
<xml_diff>
--- a/My DSA patterns Cheat Sheet.xlsx
+++ b/My DSA patterns Cheat Sheet.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programing World\DSA for Placements\dsa_with_dedication\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D438D7-EC9A-4659-A401-42CE466F414F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="368">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -60,10 +69,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/remove-duplicates-from-sorted-list/</t>
     </r>
@@ -74,10 +83,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array-ii/</t>
     </r>
@@ -94,10 +103,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/3sum/</t>
     </r>
@@ -108,10 +117,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/3sum-closest/</t>
     </r>
@@ -128,10 +137,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/subarray-product-less-than-k/</t>
     </r>
@@ -151,10 +160,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/4sum/</t>
     </r>
@@ -165,10 +174,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/backspace-string-compare/</t>
     </r>
@@ -179,10 +188,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/shortest-unsorted-continuous-subarray/</t>
     </r>
@@ -190,10 +199,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://www.ideserve.co.in/learn/minimum-length-subarray-sorting-which-results-in-sorted-array</t>
     </r>
@@ -207,10 +216,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/linked-list-cycle/</t>
     </r>
@@ -221,10 +230,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/linked-list-cycle-ii/</t>
     </r>
@@ -235,10 +244,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/happy-number/</t>
     </r>
@@ -255,10 +264,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
     </r>
@@ -269,10 +278,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/palindrome-linked-list/</t>
     </r>
@@ -283,10 +292,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/reorder-list/</t>
     </r>
@@ -297,10 +306,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/circular-array-loop/</t>
     </r>
@@ -332,10 +341,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/fruit-into-baskets/</t>
     </r>
@@ -346,10 +355,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
     </r>
@@ -360,10 +369,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/longest-repeating-character-replacement/</t>
     </r>
@@ -374,10 +383,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/max-consecutive-ones-iii/</t>
     </r>
@@ -397,10 +406,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/permutation-in-string/</t>
     </r>
@@ -411,10 +420,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/find-all-anagrams-in-a-string/</t>
     </r>
@@ -530,10 +539,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://www.geeksforgeeks.org/check-if-any-two-intervals-overlap-among-a-given-set-of-intervals/</t>
     </r>
@@ -550,10 +559,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://www.geeksforgeeks.org/maximum-cpu-load-from-the-given-list-of-jobs/</t>
     </r>
@@ -564,10 +573,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://www.codertrain.co/employee-free-time</t>
     </r>
@@ -581,10 +590,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://www.geeksforgeeks.org/sort-an-array-which-contain-1-to-n-values-in-on-using-cycle-sort/</t>
     </r>
@@ -595,10 +604,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/missing-number/</t>
     </r>
@@ -609,10 +618,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/find-all-numbers-disappeared-in-an-array/</t>
     </r>
@@ -623,10 +632,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/find-the-duplicate-number/</t>
     </r>
@@ -637,10 +646,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/find-all-duplicates-in-an-array/</t>
     </r>
@@ -651,10 +660,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://thecodingsimplified.com/find-currupt-pair/</t>
     </r>
@@ -665,10 +674,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/first-missing-positive/</t>
     </r>
@@ -679,10 +688,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://thecodingsimplified.com/find-the-first-k-missing-positive-number/</t>
     </r>
@@ -696,10 +705,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/reverse-linked-list/</t>
     </r>
@@ -710,10 +719,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/reverse-linked-list-ii/</t>
     </r>
@@ -730,10 +739,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/reverse-nodes-in-k-group/</t>
     </r>
@@ -750,10 +759,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/rotate-list/</t>
     </r>
@@ -773,10 +782,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/valid-parentheses/description/</t>
     </r>
@@ -796,10 +805,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/daily-temperatures/</t>
     </r>
@@ -810,10 +819,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/remove-nodes-from-linked-list/</t>
     </r>
@@ -824,10 +833,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/remove-all-adjacent-duplicates-in-string-ii/</t>
     </r>
@@ -844,10 +853,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/remove-k-digits/</t>
     </r>
@@ -861,10 +870,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
     </r>
@@ -875,10 +884,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/maximum-number-of-balloons/</t>
     </r>
@@ -889,10 +898,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/longest-palindrome/</t>
     </r>
@@ -903,10 +912,10 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri, sans-serif"/>
       </rPr>
       <t>https://leetcode.com/problems/ransom-note/</t>
     </r>
@@ -1480,108 +1489,122 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/serialize-and-deserialize-binary-tree/description/</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="17">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="18">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF1155CC"/>
+      <name val="Calibri, sans-serif"/>
     </font>
   </fonts>
   <fills count="12">
@@ -1589,7 +1612,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1653,7 +1676,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -1667,132 +1696,79 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="35">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="8" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="10" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="11" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1982,24 +1958,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G180"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="2" width="17.63"/>
-    <col customWidth="1" min="3" max="3" width="65.5"/>
-    <col customWidth="1" min="4" max="4" width="77.25"/>
-    <col customWidth="1" min="5" max="5" width="53.13"/>
-    <col customWidth="1" min="6" max="6" width="30.5"/>
+    <col min="1" max="2" width="17.6640625" customWidth="1"/>
+    <col min="3" max="3" width="65.44140625" customWidth="1"/>
+    <col min="4" max="4" width="77.21875" customWidth="1"/>
+    <col min="5" max="5" width="53.109375" customWidth="1"/>
+    <col min="6" max="6" width="30.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
@@ -2012,7 +1991,7 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -2032,7 +2011,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" ht="15.75" customHeight="1">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
@@ -2042,172 +2021,173 @@
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
     </row>
-    <row r="4">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="11" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
     </row>
-    <row r="5">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="7"/>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="15"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="s">
+      <c r="E5" s="13"/>
+      <c r="F5" s="14"/>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A6" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="7"/>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="7"/>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A8" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="7"/>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="12" t="s">
         <v>21</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="7"/>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="12" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A10" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="7"/>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="12" t="s">
         <v>25</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" ht="15.75" customHeight="1">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="12" t="s">
         <v>27</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A12" s="7" t="s">
         <v>28</v>
       </c>
       <c r="B12" s="7"/>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="12" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" ht="15.75" customHeight="1">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="12" t="s">
         <v>32</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" ht="15.75" customHeight="1">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="12" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" ht="15.75" customHeight="1">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="33" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="16">
+      <c r="F15" s="34"/>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" customHeight="1">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="8" t="s">
@@ -2217,103 +2197,103 @@
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="D17" s="12" t="s">
         <v>40</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="12" t="s">
         <v>42</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:6" ht="15.75" customHeight="1">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="12" t="s">
         <v>46</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="12" t="s">
         <v>48</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="12" t="s">
         <v>50</v>
       </c>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="D23" s="12" t="s">
         <v>52</v>
       </c>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="12" t="s">
         <v>54</v>
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="8" t="s">
@@ -2323,151 +2303,169 @@
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
-    <row r="26">
-      <c r="A26" s="7"/>
+    <row r="26" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A26" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B26" s="7"/>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D26" s="18" t="s">
+      <c r="D26" s="17" t="s">
         <v>57</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27">
-      <c r="A27" s="7"/>
+    <row r="27" spans="1:6" ht="14.4">
+      <c r="A27" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B27" s="7"/>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="12" t="s">
         <v>59</v>
       </c>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
     </row>
-    <row r="28">
-      <c r="A28" s="7"/>
+    <row r="28" spans="1:6" ht="14.4">
+      <c r="A28" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B28" s="7"/>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="12" t="s">
         <v>61</v>
       </c>
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
     </row>
-    <row r="29">
-      <c r="A29" s="7"/>
+    <row r="29" spans="1:6" ht="14.4">
+      <c r="A29" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B29" s="7"/>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="D29" s="12" t="s">
         <v>63</v>
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
     </row>
-    <row r="30">
-      <c r="A30" s="7"/>
+    <row r="30" spans="1:6" ht="14.4">
+      <c r="A30" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B30" s="7"/>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D30" s="12" t="s">
         <v>65</v>
       </c>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
-    <row r="31">
-      <c r="A31" s="7"/>
+    <row r="31" spans="1:6" ht="14.4">
+      <c r="A31" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B31" s="7"/>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D31" s="12" t="s">
         <v>67</v>
       </c>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
     </row>
-    <row r="32">
-      <c r="A32" s="7"/>
+    <row r="32" spans="1:6" ht="14.4">
+      <c r="A32" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B32" s="7"/>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="12" t="s">
         <v>69</v>
       </c>
       <c r="E32" s="9"/>
       <c r="F32" s="9"/>
     </row>
-    <row r="33">
-      <c r="A33" s="7"/>
+    <row r="33" spans="1:6" ht="14.4">
+      <c r="A33" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B33" s="7"/>
-      <c r="C33" s="11" t="s">
+      <c r="C33" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D33" s="12" t="s">
         <v>59</v>
       </c>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
     </row>
-    <row r="34">
-      <c r="A34" s="7"/>
+    <row r="34" spans="1:6" ht="14.4">
+      <c r="A34" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B34" s="7"/>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D34" s="12" t="s">
         <v>72</v>
       </c>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:6" ht="14.4">
       <c r="A35" s="7"/>
       <c r="B35" s="7"/>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="D35" s="12" t="s">
         <v>74</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:6" ht="14.4">
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D36" s="12" t="s">
         <v>76</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:6" ht="14.4">
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="D37" s="16" t="s">
+      <c r="D37" s="15" t="s">
         <v>78</v>
       </c>
       <c r="E37" s="9"/>
       <c r="F37" s="9"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:6" ht="14.4">
       <c r="A38" s="7"/>
       <c r="B38" s="7"/>
       <c r="C38" s="8" t="s">
@@ -2477,79 +2475,83 @@
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
     </row>
-    <row r="39">
-      <c r="A39" s="7"/>
+    <row r="39" spans="1:6" ht="14.4">
+      <c r="A39" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B39" s="7"/>
-      <c r="C39" s="19" t="s">
+      <c r="C39" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="D39" s="18" t="s">
+      <c r="D39" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
     </row>
-    <row r="40">
-      <c r="A40" s="7"/>
+    <row r="40" spans="1:6" ht="14.4">
+      <c r="A40" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="B40" s="7"/>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D40" s="18" t="s">
+      <c r="D40" s="17" t="s">
         <v>83</v>
       </c>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:6" ht="14.4">
       <c r="A41" s="7"/>
       <c r="B41" s="7"/>
-      <c r="C41" s="19" t="s">
+      <c r="C41" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="D41" s="18" t="s">
+      <c r="D41" s="17" t="s">
         <v>85</v>
       </c>
       <c r="E41" s="9"/>
       <c r="F41" s="9"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:6" ht="14.4">
       <c r="A42" s="7"/>
       <c r="B42" s="7"/>
-      <c r="C42" s="19" t="s">
+      <c r="C42" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="17" t="s">
         <v>87</v>
       </c>
       <c r="E42" s="9"/>
       <c r="F42" s="9"/>
     </row>
-    <row r="43">
+    <row r="43" spans="1:6" ht="14.4">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
-      <c r="C43" s="19" t="s">
+      <c r="C43" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="D43" s="18" t="s">
+      <c r="D43" s="17" t="s">
         <v>89</v>
       </c>
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
     </row>
-    <row r="44">
+    <row r="44" spans="1:6" ht="14.4">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
-      <c r="C44" s="19" t="s">
+      <c r="C44" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="D44" s="18" t="s">
+      <c r="D44" s="17" t="s">
         <v>91</v>
       </c>
       <c r="E44" s="9"/>
       <c r="F44" s="9"/>
     </row>
-    <row r="45">
+    <row r="45" spans="1:6" ht="14.4">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="8" t="s">
@@ -2559,79 +2561,79 @@
       <c r="E45" s="9"/>
       <c r="F45" s="9"/>
     </row>
-    <row r="46">
+    <row r="46" spans="1:6" ht="14.4">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
-      <c r="C46" s="19" t="s">
+      <c r="C46" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D46" s="18" t="s">
+      <c r="D46" s="17" t="s">
         <v>94</v>
       </c>
       <c r="E46" s="9"/>
       <c r="F46" s="9"/>
     </row>
-    <row r="47">
+    <row r="47" spans="1:6" ht="14.4">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
-      <c r="C47" s="19" t="s">
+      <c r="C47" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D47" s="18" t="s">
+      <c r="D47" s="17" t="s">
         <v>96</v>
       </c>
       <c r="E47" s="9"/>
       <c r="F47" s="9"/>
     </row>
-    <row r="48">
+    <row r="48" spans="1:6" ht="14.4">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
-      <c r="C48" s="19" t="s">
+      <c r="C48" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D48" s="18" t="s">
+      <c r="D48" s="17" t="s">
         <v>98</v>
       </c>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
     </row>
-    <row r="49">
+    <row r="49" spans="1:6" ht="14.4">
       <c r="A49" s="7"/>
       <c r="B49" s="7"/>
-      <c r="C49" s="19" t="s">
+      <c r="C49" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D49" s="18" t="s">
+      <c r="D49" s="17" t="s">
         <v>100</v>
       </c>
       <c r="E49" s="9"/>
       <c r="F49" s="9"/>
     </row>
-    <row r="50">
+    <row r="50" spans="1:6" ht="14.4">
       <c r="A50" s="7"/>
       <c r="B50" s="7"/>
-      <c r="C50" s="20" t="s">
+      <c r="C50" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="D50" s="18" t="s">
+      <c r="D50" s="17" t="s">
         <v>102</v>
       </c>
       <c r="E50" s="9"/>
       <c r="F50" s="9"/>
     </row>
-    <row r="51">
+    <row r="51" spans="1:6" ht="14.4">
       <c r="A51" s="7"/>
       <c r="B51" s="7"/>
-      <c r="C51" s="20" t="s">
+      <c r="C51" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="D51" s="18" t="s">
+      <c r="D51" s="17" t="s">
         <v>104</v>
       </c>
       <c r="E51" s="9"/>
       <c r="F51" s="9"/>
     </row>
-    <row r="52">
+    <row r="52" spans="1:6" ht="14.4">
       <c r="A52" s="7"/>
       <c r="B52" s="7"/>
       <c r="C52" s="8" t="s">
@@ -2641,90 +2643,91 @@
       <c r="E52" s="9"/>
       <c r="F52" s="9"/>
     </row>
-    <row r="53">
+    <row r="53" spans="1:6" ht="14.4">
       <c r="A53" s="7"/>
       <c r="B53" s="7"/>
-      <c r="C53" s="11" t="s">
+      <c r="C53" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D53" s="13" t="s">
+      <c r="D53" s="12" t="s">
         <v>107</v>
       </c>
       <c r="E53" s="9"/>
       <c r="F53" s="9"/>
     </row>
-    <row r="54">
+    <row r="54" spans="1:6" ht="14.4">
       <c r="A54" s="7"/>
       <c r="B54" s="7"/>
-      <c r="C54" s="11" t="s">
+      <c r="C54" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D54" s="13" t="s">
+      <c r="D54" s="12" t="s">
         <v>109</v>
       </c>
       <c r="E54" s="9"/>
       <c r="F54" s="9"/>
     </row>
-    <row r="55">
+    <row r="55" spans="1:6" ht="14.4">
       <c r="A55" s="7"/>
       <c r="B55" s="7"/>
-      <c r="C55" s="11" t="s">
+      <c r="C55" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="D55" s="13" t="s">
+      <c r="D55" s="12" t="s">
         <v>111</v>
       </c>
       <c r="E55" s="9"/>
       <c r="F55" s="9"/>
     </row>
-    <row r="56">
+    <row r="56" spans="1:6" ht="14.4">
       <c r="A56" s="7"/>
       <c r="B56" s="7"/>
-      <c r="C56" s="11" t="s">
+      <c r="C56" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D56" s="13" t="s">
+      <c r="D56" s="33" t="s">
         <v>113</v>
       </c>
+      <c r="E56" s="34"/>
       <c r="F56" s="9"/>
     </row>
-    <row r="57">
+    <row r="57" spans="1:6" ht="14.4">
       <c r="A57" s="7"/>
       <c r="B57" s="7"/>
-      <c r="C57" s="11" t="s">
+      <c r="C57" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="D57" s="13" t="s">
+      <c r="D57" s="12" t="s">
         <v>115</v>
       </c>
       <c r="E57" s="9"/>
       <c r="F57" s="9"/>
     </row>
-    <row r="58">
+    <row r="58" spans="1:6" ht="14.4">
       <c r="A58" s="7"/>
       <c r="B58" s="7"/>
-      <c r="C58" s="10" t="s">
+      <c r="C58" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D58" s="13" t="s">
+      <c r="D58" s="12" t="s">
         <v>117</v>
       </c>
       <c r="E58" s="9"/>
       <c r="F58" s="9"/>
     </row>
-    <row r="59">
+    <row r="59" spans="1:6" ht="14.4">
       <c r="A59" s="7"/>
       <c r="B59" s="7"/>
-      <c r="C59" s="10" t="s">
+      <c r="C59" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="D59" s="13" t="s">
+      <c r="D59" s="12" t="s">
         <v>119</v>
       </c>
       <c r="E59" s="9"/>
       <c r="F59" s="9"/>
     </row>
-    <row r="60">
+    <row r="60" spans="1:6" ht="14.4">
       <c r="A60" s="7"/>
       <c r="B60" s="7"/>
       <c r="C60" s="8" t="s">
@@ -2734,102 +2737,103 @@
       <c r="E60" s="9"/>
       <c r="F60" s="9"/>
     </row>
-    <row r="61">
+    <row r="61" spans="1:6" ht="14.4">
       <c r="A61" s="7"/>
       <c r="B61" s="7"/>
-      <c r="C61" s="10" t="s">
+      <c r="C61" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D61" s="13" t="s">
+      <c r="D61" s="33" t="s">
         <v>122</v>
       </c>
+      <c r="E61" s="34"/>
       <c r="F61" s="9"/>
     </row>
-    <row r="62">
+    <row r="62" spans="1:6" ht="14.4">
       <c r="A62" s="7"/>
       <c r="B62" s="7"/>
-      <c r="C62" s="10" t="s">
+      <c r="C62" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D62" s="13" t="s">
+      <c r="D62" s="12" t="s">
         <v>124</v>
       </c>
       <c r="E62" s="9"/>
       <c r="F62" s="9"/>
     </row>
-    <row r="63">
+    <row r="63" spans="1:6" ht="14.4">
       <c r="A63" s="7"/>
       <c r="B63" s="7"/>
-      <c r="C63" s="10" t="s">
+      <c r="C63" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="D63" s="13" t="s">
+      <c r="D63" s="12" t="s">
         <v>126</v>
       </c>
       <c r="E63" s="9"/>
       <c r="F63" s="9"/>
     </row>
-    <row r="64">
+    <row r="64" spans="1:6" ht="14.4">
       <c r="A64" s="7"/>
       <c r="B64" s="7"/>
-      <c r="C64" s="10" t="s">
+      <c r="C64" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="D64" s="13" t="s">
+      <c r="D64" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E64" s="9"/>
       <c r="F64" s="9"/>
     </row>
-    <row r="65">
+    <row r="65" spans="1:6" ht="14.4">
       <c r="A65" s="7"/>
       <c r="B65" s="7"/>
-      <c r="C65" s="10" t="s">
+      <c r="C65" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="D65" s="13" t="s">
+      <c r="D65" s="12" t="s">
         <v>130</v>
       </c>
       <c r="E65" s="9"/>
       <c r="F65" s="9"/>
     </row>
-    <row r="66">
+    <row r="66" spans="1:6" ht="14.4">
       <c r="A66" s="7"/>
       <c r="B66" s="7"/>
-      <c r="C66" s="10" t="s">
+      <c r="C66" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="D66" s="13" t="s">
+      <c r="D66" s="12" t="s">
         <v>132</v>
       </c>
       <c r="E66" s="9"/>
       <c r="F66" s="9"/>
     </row>
-    <row r="67">
+    <row r="67" spans="1:6" ht="14.4">
       <c r="A67" s="7"/>
       <c r="B67" s="7"/>
-      <c r="C67" s="10" t="s">
+      <c r="C67" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="D67" s="13" t="s">
+      <c r="D67" s="12" t="s">
         <v>134</v>
       </c>
       <c r="E67" s="9"/>
       <c r="F67" s="9"/>
     </row>
-    <row r="68">
+    <row r="68" spans="1:6" ht="14.4">
       <c r="A68" s="7"/>
       <c r="B68" s="7"/>
-      <c r="C68" s="10" t="s">
+      <c r="C68" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="D68" s="13" t="s">
+      <c r="D68" s="12" t="s">
         <v>136</v>
       </c>
       <c r="E68" s="9"/>
       <c r="F68" s="9"/>
     </row>
-    <row r="69">
+    <row r="69" spans="1:6" ht="14.4">
       <c r="A69" s="7"/>
       <c r="B69" s="7"/>
       <c r="C69" s="8" t="s">
@@ -2839,79 +2843,79 @@
       <c r="E69" s="9"/>
       <c r="F69" s="9"/>
     </row>
-    <row r="70">
+    <row r="70" spans="1:6" ht="14.4">
       <c r="A70" s="7"/>
       <c r="B70" s="7"/>
-      <c r="C70" s="11" t="s">
+      <c r="C70" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D70" s="13" t="s">
+      <c r="D70" s="12" t="s">
         <v>139</v>
       </c>
       <c r="E70" s="9"/>
       <c r="F70" s="9"/>
     </row>
-    <row r="71">
+    <row r="71" spans="1:6" ht="14.4">
       <c r="A71" s="7"/>
       <c r="B71" s="7"/>
-      <c r="C71" s="11" t="s">
+      <c r="C71" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D71" s="13" t="s">
+      <c r="D71" s="12" t="s">
         <v>141</v>
       </c>
       <c r="E71" s="9"/>
       <c r="F71" s="9"/>
     </row>
-    <row r="72">
+    <row r="72" spans="1:6" ht="14.4">
       <c r="A72" s="7"/>
       <c r="B72" s="7"/>
-      <c r="C72" s="11" t="s">
+      <c r="C72" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="D72" s="13" t="s">
+      <c r="D72" s="12" t="s">
         <v>143</v>
       </c>
       <c r="E72" s="9"/>
       <c r="F72" s="9"/>
     </row>
-    <row r="73">
+    <row r="73" spans="1:6" ht="14.4">
       <c r="A73" s="7"/>
       <c r="B73" s="7"/>
-      <c r="C73" s="11" t="s">
+      <c r="C73" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="D73" s="13" t="s">
+      <c r="D73" s="12" t="s">
         <v>145</v>
       </c>
       <c r="E73" s="9"/>
       <c r="F73" s="9"/>
     </row>
-    <row r="74">
+    <row r="74" spans="1:6" ht="14.4">
       <c r="A74" s="7"/>
       <c r="B74" s="7"/>
-      <c r="C74" s="10" t="s">
+      <c r="C74" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="D74" s="13" t="s">
+      <c r="D74" s="12" t="s">
         <v>147</v>
       </c>
       <c r="E74" s="9"/>
       <c r="F74" s="9"/>
     </row>
-    <row r="75">
+    <row r="75" spans="1:6" ht="14.4">
       <c r="A75" s="7"/>
       <c r="B75" s="7"/>
-      <c r="C75" s="11" t="s">
+      <c r="C75" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="D75" s="13" t="s">
+      <c r="D75" s="12" t="s">
         <v>149</v>
       </c>
       <c r="E75" s="9"/>
       <c r="F75" s="9"/>
     </row>
-    <row r="76">
+    <row r="76" spans="1:6" ht="14.4">
       <c r="A76" s="7"/>
       <c r="B76" s="7"/>
       <c r="C76" s="8" t="s">
@@ -2921,113 +2925,113 @@
       <c r="E76" s="9"/>
       <c r="F76" s="9"/>
     </row>
-    <row r="77">
+    <row r="77" spans="1:6" ht="14.4">
       <c r="A77" s="7"/>
       <c r="B77" s="7"/>
-      <c r="C77" s="21" t="s">
+      <c r="C77" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="D77" s="13" t="s">
+      <c r="D77" s="12" t="s">
         <v>152</v>
       </c>
       <c r="E77" s="9"/>
       <c r="F77" s="9"/>
     </row>
-    <row r="78">
+    <row r="78" spans="1:6" ht="14.4">
       <c r="A78" s="7"/>
       <c r="B78" s="7"/>
-      <c r="C78" s="11" t="s">
+      <c r="C78" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="D78" s="13" t="s">
+      <c r="D78" s="12" t="s">
         <v>154</v>
       </c>
       <c r="E78" s="9"/>
       <c r="F78" s="9"/>
     </row>
-    <row r="79">
+    <row r="79" spans="1:6" ht="14.4">
       <c r="A79" s="7"/>
       <c r="B79" s="7"/>
-      <c r="C79" s="11" t="s">
+      <c r="C79" s="10" t="s">
         <v>155</v>
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9"/>
       <c r="F79" s="9"/>
     </row>
-    <row r="80">
+    <row r="80" spans="1:6" ht="14.4">
       <c r="A80" s="7"/>
       <c r="B80" s="7"/>
-      <c r="C80" s="11" t="s">
+      <c r="C80" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="D80" s="13" t="s">
+      <c r="D80" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="E80" s="15"/>
-      <c r="F80" s="15"/>
-    </row>
-    <row r="81">
+      <c r="E80" s="14"/>
+      <c r="F80" s="14"/>
+    </row>
+    <row r="81" spans="1:6" ht="14.4">
       <c r="A81" s="7"/>
       <c r="B81" s="7"/>
-      <c r="C81" s="11" t="s">
+      <c r="C81" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="D81" s="13" t="s">
+      <c r="D81" s="12" t="s">
         <v>159</v>
       </c>
       <c r="E81" s="9"/>
       <c r="F81" s="9"/>
     </row>
-    <row r="82">
+    <row r="82" spans="1:6" ht="14.4">
       <c r="A82" s="7"/>
       <c r="B82" s="7"/>
-      <c r="C82" s="10" t="s">
+      <c r="C82" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="D82" s="13" t="s">
+      <c r="D82" s="12" t="s">
         <v>161</v>
       </c>
       <c r="E82" s="9"/>
       <c r="F82" s="9"/>
     </row>
-    <row r="83">
+    <row r="83" spans="1:6" ht="14.4">
       <c r="A83" s="7"/>
       <c r="B83" s="7"/>
-      <c r="C83" s="11" t="s">
+      <c r="C83" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="D83" s="13" t="s">
+      <c r="D83" s="12" t="s">
         <v>163</v>
       </c>
       <c r="E83" s="9"/>
       <c r="F83" s="9"/>
     </row>
-    <row r="84">
+    <row r="84" spans="1:6" ht="14.4">
       <c r="A84" s="7"/>
       <c r="B84" s="7"/>
-      <c r="C84" s="10" t="s">
+      <c r="C84" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="D84" s="13" t="s">
+      <c r="D84" s="12" t="s">
         <v>165</v>
       </c>
       <c r="E84" s="9"/>
       <c r="F84" s="9"/>
     </row>
-    <row r="85">
+    <row r="85" spans="1:6" ht="14.4">
       <c r="A85" s="7"/>
       <c r="B85" s="7"/>
-      <c r="C85" s="10" t="s">
+      <c r="C85" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D85" s="13" t="s">
+      <c r="D85" s="12" t="s">
         <v>167</v>
       </c>
       <c r="E85" s="9"/>
       <c r="F85" s="9"/>
     </row>
-    <row r="86">
+    <row r="86" spans="1:6" ht="14.4">
       <c r="A86" s="7"/>
       <c r="B86" s="7"/>
       <c r="C86" s="8" t="s">
@@ -3037,341 +3041,341 @@
       <c r="E86" s="9"/>
       <c r="F86" s="9"/>
     </row>
-    <row r="87">
+    <row r="87" spans="1:6" ht="14.4">
       <c r="A87" s="7"/>
       <c r="B87" s="7"/>
-      <c r="C87" s="11" t="s">
+      <c r="C87" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="D87" s="13" t="s">
+      <c r="D87" s="12" t="s">
         <v>170</v>
       </c>
       <c r="E87" s="9"/>
       <c r="F87" s="9"/>
     </row>
-    <row r="88">
+    <row r="88" spans="1:6" ht="14.4">
       <c r="A88" s="7"/>
       <c r="B88" s="7"/>
-      <c r="C88" s="11" t="s">
+      <c r="C88" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="D88" s="13" t="s">
+      <c r="D88" s="12" t="s">
         <v>172</v>
       </c>
       <c r="E88" s="9"/>
       <c r="F88" s="9"/>
     </row>
-    <row r="89">
+    <row r="89" spans="1:6" ht="14.4">
       <c r="A89" s="7"/>
       <c r="B89" s="7"/>
-      <c r="C89" s="11" t="s">
+      <c r="C89" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="D89" s="13" t="s">
+      <c r="D89" s="12" t="s">
         <v>174</v>
       </c>
       <c r="E89" s="9"/>
       <c r="F89" s="9"/>
     </row>
-    <row r="90">
+    <row r="90" spans="1:6" ht="14.4">
       <c r="A90" s="7"/>
       <c r="B90" s="7"/>
-      <c r="C90" s="11" t="s">
+      <c r="C90" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="D90" s="13" t="s">
+      <c r="D90" s="12" t="s">
         <v>176</v>
       </c>
       <c r="E90" s="9"/>
       <c r="F90" s="9"/>
     </row>
-    <row r="91">
+    <row r="91" spans="1:6" ht="14.4">
       <c r="A91" s="7"/>
       <c r="B91" s="7"/>
       <c r="C91" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="D91" s="22"/>
+      <c r="D91" s="21"/>
       <c r="E91" s="9"/>
       <c r="F91" s="9"/>
     </row>
-    <row r="92">
+    <row r="92" spans="1:6" ht="14.4">
       <c r="A92" s="7"/>
       <c r="B92" s="7"/>
-      <c r="C92" s="11" t="s">
+      <c r="C92" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="D92" s="13" t="s">
+      <c r="D92" s="12" t="s">
         <v>179</v>
       </c>
       <c r="E92" s="9"/>
       <c r="F92" s="9"/>
     </row>
-    <row r="93">
+    <row r="93" spans="1:6" ht="14.4">
       <c r="A93" s="7"/>
       <c r="B93" s="7"/>
-      <c r="C93" s="11" t="s">
+      <c r="C93" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="D93" s="13" t="s">
+      <c r="D93" s="12" t="s">
         <v>181</v>
       </c>
       <c r="E93" s="9"/>
       <c r="F93" s="9"/>
     </row>
-    <row r="94">
+    <row r="94" spans="1:6" ht="14.4">
       <c r="A94" s="7"/>
       <c r="B94" s="7"/>
-      <c r="C94" s="11" t="s">
+      <c r="C94" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="D94" s="13" t="s">
+      <c r="D94" s="12" t="s">
         <v>183</v>
       </c>
       <c r="E94" s="9"/>
       <c r="F94" s="9"/>
     </row>
-    <row r="95">
+    <row r="95" spans="1:6" ht="14.4">
       <c r="A95" s="7"/>
       <c r="B95" s="7"/>
-      <c r="C95" s="11" t="s">
+      <c r="C95" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="D95" s="13" t="s">
+      <c r="D95" s="12" t="s">
         <v>185</v>
       </c>
       <c r="E95" s="9"/>
       <c r="F95" s="9"/>
     </row>
-    <row r="96">
+    <row r="96" spans="1:6" ht="14.4">
       <c r="A96" s="7"/>
       <c r="B96" s="7"/>
-      <c r="C96" s="10" t="s">
+      <c r="C96" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="D96" s="13" t="s">
+      <c r="D96" s="12" t="s">
         <v>187</v>
       </c>
       <c r="E96" s="9"/>
       <c r="F96" s="9"/>
     </row>
-    <row r="97">
+    <row r="97" spans="1:6" ht="14.4">
       <c r="A97" s="7"/>
       <c r="B97" s="7"/>
-      <c r="C97" s="11" t="s">
+      <c r="C97" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="D97" s="13" t="s">
+      <c r="D97" s="12" t="s">
         <v>189</v>
       </c>
       <c r="E97" s="9"/>
       <c r="F97" s="9"/>
     </row>
-    <row r="98">
+    <row r="98" spans="1:6" ht="14.4">
       <c r="A98" s="7"/>
       <c r="B98" s="7"/>
-      <c r="C98" s="10" t="s">
+      <c r="C98" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="D98" s="13" t="s">
+      <c r="D98" s="12" t="s">
         <v>191</v>
       </c>
       <c r="E98" s="9"/>
       <c r="F98" s="9"/>
     </row>
-    <row r="99">
+    <row r="99" spans="1:6" ht="14.4">
       <c r="A99" s="7"/>
       <c r="B99" s="7"/>
-      <c r="C99" s="11" t="s">
+      <c r="C99" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="D99" s="13" t="s">
+      <c r="D99" s="12" t="s">
         <v>193</v>
       </c>
       <c r="E99" s="9"/>
       <c r="F99" s="9"/>
     </row>
-    <row r="100">
+    <row r="100" spans="1:6" ht="14.4">
       <c r="A100" s="7"/>
       <c r="B100" s="7"/>
-      <c r="C100" s="11" t="s">
+      <c r="C100" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="D100" s="13" t="s">
+      <c r="D100" s="12" t="s">
         <v>195</v>
       </c>
       <c r="E100" s="9"/>
       <c r="F100" s="9"/>
     </row>
-    <row r="101">
+    <row r="101" spans="1:6" ht="14.4">
       <c r="A101" s="7"/>
       <c r="B101" s="7"/>
-      <c r="C101" s="11" t="s">
+      <c r="C101" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="D101" s="13" t="s">
+      <c r="D101" s="12" t="s">
         <v>197</v>
       </c>
       <c r="E101" s="9"/>
       <c r="F101" s="9"/>
     </row>
-    <row r="102">
+    <row r="102" spans="1:6" ht="14.4">
       <c r="A102" s="7"/>
       <c r="B102" s="7"/>
-      <c r="C102" s="11" t="s">
+      <c r="C102" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="D102" s="13" t="s">
+      <c r="D102" s="12" t="s">
         <v>199</v>
       </c>
       <c r="E102" s="9"/>
       <c r="F102" s="9"/>
     </row>
-    <row r="103">
+    <row r="103" spans="1:6" ht="14.4">
       <c r="A103" s="7"/>
       <c r="B103" s="7"/>
-      <c r="C103" s="10" t="s">
+      <c r="C103" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="D103" s="13" t="s">
+      <c r="D103" s="12" t="s">
         <v>201</v>
       </c>
       <c r="E103" s="9"/>
       <c r="F103" s="9"/>
     </row>
-    <row r="104">
+    <row r="104" spans="1:6" ht="14.4">
       <c r="A104" s="7"/>
       <c r="B104" s="7"/>
-      <c r="C104" s="11" t="s">
+      <c r="C104" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="D104" s="13" t="s">
+      <c r="D104" s="12" t="s">
         <v>203</v>
       </c>
       <c r="E104" s="9"/>
       <c r="F104" s="9"/>
     </row>
-    <row r="105">
+    <row r="105" spans="1:6" ht="14.4">
       <c r="A105" s="7"/>
       <c r="B105" s="7"/>
-      <c r="C105" s="23" t="s">
+      <c r="C105" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="D105" s="13" t="s">
+      <c r="D105" s="12" t="s">
         <v>205</v>
       </c>
       <c r="E105" s="9"/>
       <c r="F105" s="9"/>
     </row>
-    <row r="106">
+    <row r="106" spans="1:6" ht="14.4">
       <c r="A106" s="7"/>
       <c r="B106" s="7"/>
-      <c r="C106" s="10" t="s">
+      <c r="C106" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="D106" s="13" t="s">
+      <c r="D106" s="12" t="s">
         <v>207</v>
       </c>
       <c r="E106" s="9"/>
       <c r="F106" s="9"/>
     </row>
-    <row r="107">
+    <row r="107" spans="1:6" ht="14.4">
       <c r="A107" s="7"/>
       <c r="B107" s="7"/>
-      <c r="C107" s="10" t="s">
+      <c r="C107" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="D107" s="13" t="s">
+      <c r="D107" s="12" t="s">
         <v>209</v>
       </c>
       <c r="E107" s="9"/>
       <c r="F107" s="9"/>
     </row>
-    <row r="108">
+    <row r="108" spans="1:6" ht="14.4">
       <c r="A108" s="7"/>
       <c r="B108" s="7"/>
-      <c r="C108" s="11" t="s">
+      <c r="C108" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="D108" s="16" t="s">
+      <c r="D108" s="15" t="s">
         <v>211</v>
       </c>
       <c r="E108" s="9"/>
       <c r="F108" s="9"/>
     </row>
-    <row r="109">
+    <row r="109" spans="1:6" ht="14.4">
       <c r="A109" s="7"/>
       <c r="B109" s="7"/>
-      <c r="C109" s="10" t="s">
+      <c r="C109" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="D109" s="16" t="s">
+      <c r="D109" s="15" t="s">
         <v>213</v>
       </c>
       <c r="E109" s="9"/>
       <c r="F109" s="9"/>
     </row>
-    <row r="110">
+    <row r="110" spans="1:6" ht="14.4">
       <c r="A110" s="7"/>
       <c r="B110" s="7"/>
-      <c r="C110" s="11" t="s">
+      <c r="C110" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="D110" s="16" t="s">
+      <c r="D110" s="15" t="s">
         <v>215</v>
       </c>
       <c r="E110" s="9"/>
       <c r="F110" s="9"/>
     </row>
-    <row r="111">
+    <row r="111" spans="1:6" ht="14.4">
       <c r="A111" s="7"/>
       <c r="B111" s="7"/>
-      <c r="C111" s="11" t="s">
+      <c r="C111" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="D111" s="16" t="s">
+      <c r="D111" s="15" t="s">
         <v>217</v>
       </c>
       <c r="E111" s="9"/>
       <c r="F111" s="9"/>
     </row>
-    <row r="112">
+    <row r="112" spans="1:6" ht="14.4">
       <c r="A112" s="7"/>
       <c r="B112" s="7"/>
-      <c r="C112" s="11" t="s">
+      <c r="C112" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="D112" s="16" t="s">
+      <c r="D112" s="15" t="s">
         <v>219</v>
       </c>
       <c r="E112" s="9"/>
       <c r="F112" s="9"/>
     </row>
-    <row r="113">
+    <row r="113" spans="1:6" ht="14.4">
       <c r="A113" s="7"/>
       <c r="B113" s="7"/>
-      <c r="C113" s="11" t="s">
+      <c r="C113" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="D113" s="16" t="s">
+      <c r="D113" s="15" t="s">
         <v>221</v>
       </c>
       <c r="E113" s="9"/>
       <c r="F113" s="9"/>
     </row>
-    <row r="114">
+    <row r="114" spans="1:6" ht="14.4">
       <c r="A114" s="7"/>
       <c r="B114" s="7"/>
-      <c r="C114" s="10" t="s">
+      <c r="C114" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="D114" s="16" t="s">
+      <c r="D114" s="15" t="s">
         <v>223</v>
       </c>
       <c r="E114" s="9"/>
       <c r="F114" s="9"/>
     </row>
-    <row r="115">
+    <row r="115" spans="1:6" ht="14.4">
       <c r="A115" s="7"/>
       <c r="B115" s="7"/>
       <c r="C115" s="8" t="s">
@@ -3381,221 +3385,221 @@
       <c r="E115" s="9"/>
       <c r="F115" s="9"/>
     </row>
-    <row r="116">
-      <c r="A116" s="24"/>
-      <c r="B116" s="24" t="s">
+    <row r="116" spans="1:6" ht="14.4">
+      <c r="A116" s="23"/>
+      <c r="B116" s="23" t="s">
         <v>225</v>
       </c>
-      <c r="C116" s="25" t="s">
+      <c r="C116" s="24" t="s">
         <v>226</v>
       </c>
-      <c r="D116" s="26" t="s">
+      <c r="D116" s="25" t="s">
         <v>227</v>
       </c>
       <c r="E116" s="9"/>
       <c r="F116" s="9"/>
     </row>
-    <row r="117">
+    <row r="117" spans="1:6" ht="14.4">
       <c r="A117" s="7"/>
       <c r="B117" s="7"/>
-      <c r="C117" s="25" t="s">
+      <c r="C117" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="D117" s="26" t="s">
+      <c r="D117" s="25" t="s">
         <v>229</v>
       </c>
       <c r="E117" s="9"/>
       <c r="F117" s="9"/>
     </row>
-    <row r="118">
+    <row r="118" spans="1:6" ht="14.4">
       <c r="A118" s="7"/>
       <c r="B118" s="7"/>
-      <c r="C118" s="25" t="s">
+      <c r="C118" s="24" t="s">
         <v>230</v>
       </c>
-      <c r="D118" s="26" t="s">
+      <c r="D118" s="25" t="s">
         <v>231</v>
       </c>
       <c r="E118" s="9"/>
       <c r="F118" s="9"/>
     </row>
-    <row r="119">
+    <row r="119" spans="1:6" ht="14.4">
       <c r="A119" s="7"/>
       <c r="B119" s="7"/>
-      <c r="C119" s="25" t="s">
+      <c r="C119" s="24" t="s">
         <v>232</v>
       </c>
-      <c r="D119" s="26" t="s">
+      <c r="D119" s="25" t="s">
         <v>233</v>
       </c>
       <c r="E119" s="9"/>
       <c r="F119" s="9"/>
     </row>
-    <row r="120">
-      <c r="A120" s="24"/>
-      <c r="B120" s="24" t="s">
+    <row r="120" spans="1:6" ht="14.4">
+      <c r="A120" s="23"/>
+      <c r="B120" s="23" t="s">
         <v>234</v>
       </c>
-      <c r="C120" s="27" t="s">
+      <c r="C120" s="26" t="s">
         <v>235</v>
       </c>
-      <c r="D120" s="26" t="s">
+      <c r="D120" s="25" t="s">
         <v>236</v>
       </c>
       <c r="E120" s="9"/>
       <c r="F120" s="9"/>
     </row>
-    <row r="121">
+    <row r="121" spans="1:6" ht="14.4">
       <c r="A121" s="7"/>
       <c r="B121" s="7"/>
-      <c r="C121" s="27" t="s">
+      <c r="C121" s="26" t="s">
         <v>237</v>
       </c>
-      <c r="D121" s="18" t="s">
+      <c r="D121" s="17" t="s">
         <v>238</v>
       </c>
       <c r="E121" s="9"/>
       <c r="F121" s="9"/>
     </row>
-    <row r="122">
+    <row r="122" spans="1:6" ht="14.4">
       <c r="A122" s="7"/>
       <c r="B122" s="7"/>
-      <c r="C122" s="27" t="s">
+      <c r="C122" s="26" t="s">
         <v>239</v>
       </c>
-      <c r="D122" s="18" t="s">
+      <c r="D122" s="17" t="s">
         <v>240</v>
       </c>
       <c r="E122" s="9"/>
       <c r="F122" s="9"/>
     </row>
-    <row r="123">
-      <c r="A123" s="24"/>
-      <c r="B123" s="24" t="s">
+    <row r="123" spans="1:6" ht="14.4">
+      <c r="A123" s="23"/>
+      <c r="B123" s="23" t="s">
         <v>241</v>
       </c>
-      <c r="C123" s="28" t="s">
+      <c r="C123" s="27" t="s">
         <v>242</v>
       </c>
-      <c r="D123" s="26" t="s">
+      <c r="D123" s="25" t="s">
         <v>243</v>
       </c>
       <c r="E123" s="9"/>
       <c r="F123" s="9"/>
     </row>
-    <row r="124">
+    <row r="124" spans="1:6" ht="14.4">
       <c r="A124" s="7"/>
       <c r="B124" s="7"/>
-      <c r="C124" s="28" t="s">
+      <c r="C124" s="27" t="s">
         <v>244</v>
       </c>
-      <c r="D124" s="18" t="s">
+      <c r="D124" s="17" t="s">
         <v>219</v>
       </c>
       <c r="E124" s="9"/>
       <c r="F124" s="9"/>
     </row>
-    <row r="125">
-      <c r="A125" s="24"/>
-      <c r="B125" s="24" t="s">
+    <row r="125" spans="1:6" ht="14.4">
+      <c r="A125" s="23"/>
+      <c r="B125" s="23" t="s">
         <v>245</v>
       </c>
-      <c r="C125" s="29" t="s">
+      <c r="C125" s="28" t="s">
         <v>246</v>
       </c>
-      <c r="D125" s="18" t="s">
+      <c r="D125" s="17" t="s">
         <v>247</v>
       </c>
       <c r="E125" s="9"/>
       <c r="F125" s="9"/>
     </row>
-    <row r="126">
-      <c r="A126" s="17"/>
-      <c r="B126" s="17"/>
-      <c r="C126" s="29" t="s">
+    <row r="126" spans="1:6" ht="14.4">
+      <c r="A126" s="16"/>
+      <c r="B126" s="16"/>
+      <c r="C126" s="28" t="s">
         <v>248</v>
       </c>
-      <c r="D126" s="26" t="s">
+      <c r="D126" s="25" t="s">
         <v>249</v>
       </c>
       <c r="E126" s="9"/>
       <c r="F126" s="9"/>
     </row>
-    <row r="127">
+    <row r="127" spans="1:6" ht="14.4">
       <c r="A127" s="7"/>
       <c r="B127" s="7"/>
-      <c r="C127" s="29" t="s">
+      <c r="C127" s="28" t="s">
         <v>250</v>
       </c>
-      <c r="D127" s="26" t="s">
+      <c r="D127" s="25" t="s">
         <v>251</v>
       </c>
       <c r="E127" s="9"/>
       <c r="F127" s="9"/>
     </row>
-    <row r="128">
+    <row r="128" spans="1:6" ht="14.4">
       <c r="A128" s="7"/>
       <c r="B128" s="7"/>
-      <c r="C128" s="29" t="s">
+      <c r="C128" s="28" t="s">
         <v>252</v>
       </c>
-      <c r="D128" s="18" t="s">
+      <c r="D128" s="17" t="s">
         <v>253</v>
       </c>
       <c r="E128" s="9"/>
       <c r="F128" s="9"/>
     </row>
-    <row r="129">
+    <row r="129" spans="1:6" ht="14.4">
       <c r="A129" s="7"/>
       <c r="B129" s="7"/>
-      <c r="C129" s="29" t="s">
+      <c r="C129" s="28" t="s">
         <v>254</v>
       </c>
-      <c r="D129" s="26" t="s">
+      <c r="D129" s="25" t="s">
         <v>255</v>
       </c>
       <c r="E129" s="9"/>
       <c r="F129" s="9"/>
     </row>
-    <row r="130">
+    <row r="130" spans="1:6" ht="14.4">
       <c r="A130" s="7"/>
       <c r="B130" s="7"/>
-      <c r="C130" s="29" t="s">
+      <c r="C130" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="D130" s="18" t="s">
+      <c r="D130" s="17" t="s">
         <v>257</v>
       </c>
       <c r="E130" s="9"/>
       <c r="F130" s="9"/>
     </row>
-    <row r="131">
-      <c r="A131" s="24"/>
-      <c r="B131" s="24" t="s">
+    <row r="131" spans="1:6" ht="14.4">
+      <c r="A131" s="23"/>
+      <c r="B131" s="23" t="s">
         <v>258</v>
       </c>
-      <c r="C131" s="30" t="s">
+      <c r="C131" s="29" t="s">
         <v>259</v>
       </c>
-      <c r="D131" s="18" t="s">
+      <c r="D131" s="17" t="s">
         <v>260</v>
       </c>
       <c r="E131" s="9"/>
       <c r="F131" s="9"/>
     </row>
-    <row r="132">
+    <row r="132" spans="1:6" ht="14.4">
       <c r="A132" s="7"/>
       <c r="B132" s="7"/>
-      <c r="C132" s="30" t="s">
+      <c r="C132" s="29" t="s">
         <v>261</v>
       </c>
-      <c r="D132" s="18" t="s">
+      <c r="D132" s="17" t="s">
         <v>262</v>
       </c>
       <c r="E132" s="9"/>
       <c r="F132" s="9"/>
     </row>
-    <row r="133">
+    <row r="133" spans="1:6" ht="14.4">
       <c r="A133" s="7"/>
       <c r="B133" s="7"/>
       <c r="C133" s="8" t="s">
@@ -3605,461 +3609,461 @@
       <c r="E133" s="9"/>
       <c r="F133" s="9"/>
     </row>
-    <row r="134">
+    <row r="134" spans="1:6" ht="14.4">
       <c r="A134" s="7"/>
       <c r="B134" s="7"/>
-      <c r="C134" s="11" t="s">
+      <c r="C134" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="D134" s="26" t="s">
+      <c r="D134" s="25" t="s">
         <v>265</v>
       </c>
-      <c r="E134" s="18" t="s">
+      <c r="E134" s="17" t="s">
         <v>266</v>
       </c>
       <c r="F134" s="9"/>
     </row>
-    <row r="135">
+    <row r="135" spans="1:6" ht="14.4">
       <c r="A135" s="7"/>
       <c r="B135" s="7"/>
-      <c r="C135" s="11" t="s">
+      <c r="C135" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="D135" s="26" t="s">
+      <c r="D135" s="25" t="s">
         <v>268</v>
       </c>
-      <c r="E135" s="18" t="s">
+      <c r="E135" s="17" t="s">
         <v>266</v>
       </c>
       <c r="F135" s="9"/>
     </row>
-    <row r="136">
+    <row r="136" spans="1:6" ht="14.4">
       <c r="A136" s="7"/>
       <c r="B136" s="7"/>
-      <c r="C136" s="11" t="s">
+      <c r="C136" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="D136" s="26" t="s">
+      <c r="D136" s="25" t="s">
         <v>270</v>
       </c>
-      <c r="E136" s="18" t="s">
+      <c r="E136" s="17" t="s">
         <v>271</v>
       </c>
       <c r="F136" s="9"/>
     </row>
-    <row r="137">
+    <row r="137" spans="1:6" ht="14.4">
       <c r="A137" s="7"/>
       <c r="B137" s="7"/>
-      <c r="C137" s="11" t="s">
+      <c r="C137" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="D137" s="26" t="s">
+      <c r="D137" s="25" t="s">
         <v>273</v>
       </c>
-      <c r="E137" s="18" t="s">
+      <c r="E137" s="17" t="s">
         <v>271</v>
       </c>
       <c r="F137" s="9"/>
     </row>
-    <row r="138">
+    <row r="138" spans="1:6" ht="14.4">
       <c r="A138" s="7"/>
       <c r="B138" s="7"/>
-      <c r="C138" s="11" t="s">
+      <c r="C138" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="D138" s="26" t="s">
+      <c r="D138" s="25" t="s">
         <v>275</v>
       </c>
-      <c r="E138" s="18" t="s">
+      <c r="E138" s="17" t="s">
         <v>271</v>
       </c>
       <c r="F138" s="9"/>
     </row>
-    <row r="139">
+    <row r="139" spans="1:6" ht="14.4">
       <c r="A139" s="7"/>
       <c r="B139" s="7"/>
-      <c r="C139" s="11" t="s">
+      <c r="C139" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="D139" s="26" t="s">
+      <c r="D139" s="25" t="s">
         <v>277</v>
       </c>
       <c r="E139" s="9"/>
       <c r="F139" s="9"/>
     </row>
-    <row r="140">
+    <row r="140" spans="1:6" ht="14.4">
       <c r="A140" s="7"/>
       <c r="B140" s="7"/>
-      <c r="C140" s="11" t="s">
+      <c r="C140" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="D140" s="26" t="s">
+      <c r="D140" s="25" t="s">
         <v>279</v>
       </c>
-      <c r="E140" s="18" t="s">
+      <c r="E140" s="17" t="s">
         <v>280</v>
       </c>
       <c r="F140" s="9"/>
     </row>
-    <row r="141">
+    <row r="141" spans="1:6" ht="14.4">
       <c r="A141" s="7"/>
       <c r="B141" s="7"/>
-      <c r="C141" s="11" t="s">
+      <c r="C141" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="D141" s="18" t="s">
+      <c r="D141" s="17" t="s">
         <v>282</v>
       </c>
       <c r="E141" s="9"/>
       <c r="F141" s="9"/>
     </row>
-    <row r="142">
+    <row r="142" spans="1:6" ht="14.4">
       <c r="A142" s="7"/>
       <c r="B142" s="7"/>
-      <c r="C142" s="11" t="s">
+      <c r="C142" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="D142" s="26" t="s">
+      <c r="D142" s="25" t="s">
         <v>284</v>
       </c>
       <c r="E142" s="9"/>
       <c r="F142" s="9"/>
     </row>
-    <row r="143">
+    <row r="143" spans="1:6" ht="14.4">
       <c r="A143" s="7"/>
       <c r="B143" s="7"/>
-      <c r="C143" s="17" t="s">
+      <c r="C143" s="16" t="s">
         <v>285</v>
       </c>
-      <c r="D143" s="18" t="s">
+      <c r="D143" s="17" t="s">
         <v>286</v>
       </c>
       <c r="E143" s="9"/>
       <c r="F143" s="9"/>
     </row>
-    <row r="144">
+    <row r="144" spans="1:6" ht="14.4">
       <c r="C144" s="8" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="19"/>
-      <c r="B145" s="19" t="s">
+    <row r="145" spans="1:5" ht="13.2">
+      <c r="A145" s="18"/>
+      <c r="B145" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="C145" s="20" t="s">
+      <c r="C145" s="19" t="s">
         <v>289</v>
       </c>
-      <c r="D145" s="31" t="s">
+      <c r="D145" s="30" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="146">
-      <c r="C146" s="20" t="s">
+    <row r="146" spans="1:5" ht="13.2">
+      <c r="C146" s="19" t="s">
         <v>291</v>
       </c>
-      <c r="D146" s="31" t="s">
+      <c r="D146" s="30" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="147">
-      <c r="C147" s="20" t="s">
+    <row r="147" spans="1:5" ht="13.2">
+      <c r="C147" s="19" t="s">
         <v>293</v>
       </c>
-      <c r="D147" s="31" t="s">
+      <c r="D147" s="30" t="s">
         <v>294</v>
       </c>
-      <c r="E147" s="20" t="s">
+      <c r="E147" s="19" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="148">
-      <c r="C148" s="20" t="s">
+    <row r="148" spans="1:5" ht="13.2">
+      <c r="C148" s="19" t="s">
         <v>296</v>
       </c>
-      <c r="D148" s="31" t="s">
+      <c r="D148" s="30" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="149">
-      <c r="C149" s="20" t="s">
+    <row r="149" spans="1:5" ht="13.2">
+      <c r="C149" s="19" t="s">
         <v>298</v>
       </c>
-      <c r="D149" s="31" t="s">
+      <c r="D149" s="30" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="150">
-      <c r="C150" s="20" t="s">
+    <row r="150" spans="1:5" ht="13.2">
+      <c r="C150" s="19" t="s">
         <v>300</v>
       </c>
-      <c r="D150" s="31" t="s">
+      <c r="D150" s="30" t="s">
         <v>301</v>
       </c>
-      <c r="E150" s="20" t="s">
+      <c r="E150" s="19" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="32"/>
-      <c r="B151" s="32" t="s">
+    <row r="151" spans="1:5" ht="13.2">
+      <c r="A151" s="31"/>
+      <c r="B151" s="31" t="s">
         <v>302</v>
       </c>
-      <c r="C151" s="20" t="s">
+      <c r="C151" s="19" t="s">
         <v>303</v>
       </c>
-      <c r="D151" s="31" t="s">
+      <c r="D151" s="30" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="152">
-      <c r="C152" s="20" t="s">
+    <row r="152" spans="1:5" ht="13.2">
+      <c r="C152" s="19" t="s">
         <v>305</v>
       </c>
-      <c r="D152" s="31" t="s">
+      <c r="D152" s="30" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="153">
-      <c r="C153" s="20" t="s">
+    <row r="153" spans="1:5" ht="13.2">
+      <c r="C153" s="19" t="s">
         <v>307</v>
       </c>
-      <c r="D153" s="31" t="s">
+      <c r="D153" s="30" t="s">
         <v>308</v>
       </c>
-      <c r="E153" s="20" t="s">
+      <c r="E153" s="19" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="154">
-      <c r="C154" s="20" t="s">
+    <row r="154" spans="1:5" ht="13.2">
+      <c r="C154" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="D154" s="33" t="s">
+      <c r="D154" s="32" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="155">
-      <c r="C155" s="20" t="s">
+    <row r="155" spans="1:5" ht="13.2">
+      <c r="C155" s="19" t="s">
         <v>311</v>
       </c>
-      <c r="D155" s="33" t="s">
+      <c r="D155" s="32" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="32"/>
-      <c r="B156" s="32" t="s">
+    <row r="156" spans="1:5" ht="13.2">
+      <c r="A156" s="31"/>
+      <c r="B156" s="31" t="s">
         <v>313</v>
       </c>
-      <c r="C156" s="20" t="s">
+      <c r="C156" s="19" t="s">
         <v>314</v>
       </c>
-      <c r="D156" s="31" t="s">
+      <c r="D156" s="30" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="157">
-      <c r="C157" s="20" t="s">
+    <row r="157" spans="1:5" ht="13.2">
+      <c r="C157" s="19" t="s">
         <v>316</v>
       </c>
-      <c r="D157" s="31" t="s">
+      <c r="D157" s="30" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="158">
-      <c r="C158" s="20" t="s">
+    <row r="158" spans="1:5" ht="13.2">
+      <c r="C158" s="19" t="s">
         <v>318</v>
       </c>
-      <c r="D158" s="33" t="s">
+      <c r="D158" s="32" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="159">
-      <c r="C159" s="20" t="s">
+    <row r="159" spans="1:5" ht="13.2">
+      <c r="C159" s="19" t="s">
         <v>320</v>
       </c>
-      <c r="D159" s="33" t="s">
+      <c r="D159" s="32" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="160">
-      <c r="C160" s="20" t="s">
+    <row r="160" spans="1:5" ht="13.2">
+      <c r="C160" s="19" t="s">
         <v>322</v>
       </c>
-      <c r="D160" s="33" t="s">
+      <c r="D160" s="32" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="161">
-      <c r="C161" s="20" t="s">
+    <row r="161" spans="1:4" ht="13.2">
+      <c r="C161" s="19" t="s">
         <v>324</v>
       </c>
-      <c r="D161" s="33" t="s">
+      <c r="D161" s="32" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="162">
-      <c r="A162" s="32"/>
-      <c r="B162" s="32" t="s">
+    <row r="162" spans="1:4" ht="13.2">
+      <c r="A162" s="31"/>
+      <c r="B162" s="31" t="s">
         <v>326</v>
       </c>
-      <c r="C162" s="20" t="s">
+      <c r="C162" s="19" t="s">
         <v>327</v>
       </c>
-      <c r="D162" s="33" t="s">
+      <c r="D162" s="32" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="163">
-      <c r="C163" s="20" t="s">
+    <row r="163" spans="1:4" ht="13.2">
+      <c r="C163" s="19" t="s">
         <v>329</v>
       </c>
-      <c r="D163" s="33" t="s">
+      <c r="D163" s="32" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="164">
-      <c r="C164" s="20" t="s">
+    <row r="164" spans="1:4" ht="13.2">
+      <c r="C164" s="19" t="s">
         <v>331</v>
       </c>
-      <c r="D164" s="33" t="s">
+      <c r="D164" s="32" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="165">
-      <c r="C165" s="20" t="s">
+    <row r="165" spans="1:4" ht="13.2">
+      <c r="C165" s="19" t="s">
         <v>333</v>
       </c>
-      <c r="D165" s="33" t="s">
+      <c r="D165" s="32" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="166">
-      <c r="C166" s="20" t="s">
+    <row r="166" spans="1:4" ht="13.2">
+      <c r="C166" s="19" t="s">
         <v>335</v>
       </c>
-      <c r="D166" s="33" t="s">
+      <c r="D166" s="32" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="167">
-      <c r="C167" s="20" t="s">
+    <row r="167" spans="1:4" ht="13.2">
+      <c r="C167" s="19" t="s">
         <v>337</v>
       </c>
-      <c r="D167" s="33" t="s">
+      <c r="D167" s="32" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="168">
-      <c r="C168" s="20" t="s">
+    <row r="168" spans="1:4" ht="13.2">
+      <c r="C168" s="19" t="s">
         <v>339</v>
       </c>
-      <c r="D168" s="33" t="s">
+      <c r="D168" s="32" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="169">
-      <c r="C169" s="20" t="s">
+    <row r="169" spans="1:4" ht="13.2">
+      <c r="C169" s="19" t="s">
         <v>341</v>
       </c>
-      <c r="D169" s="33" t="s">
+      <c r="D169" s="32" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="170">
-      <c r="A170" s="32"/>
-      <c r="B170" s="32" t="s">
+    <row r="170" spans="1:4" ht="13.2">
+      <c r="A170" s="31"/>
+      <c r="B170" s="31" t="s">
         <v>343</v>
       </c>
-      <c r="C170" s="20" t="s">
+      <c r="C170" s="19" t="s">
         <v>344</v>
       </c>
-      <c r="D170" s="33" t="s">
+      <c r="D170" s="32" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="171">
-      <c r="C171" s="20" t="s">
+    <row r="171" spans="1:4" ht="13.2">
+      <c r="C171" s="19" t="s">
         <v>346</v>
       </c>
-      <c r="D171" s="33" t="s">
+      <c r="D171" s="32" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="172">
-      <c r="C172" s="20" t="s">
+    <row r="172" spans="1:4" ht="13.2">
+      <c r="C172" s="19" t="s">
         <v>348</v>
       </c>
-      <c r="D172" s="33" t="s">
+      <c r="D172" s="32" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="173">
-      <c r="C173" s="20" t="s">
+    <row r="173" spans="1:4" ht="13.2">
+      <c r="C173" s="19" t="s">
         <v>350</v>
       </c>
-      <c r="D173" s="33" t="s">
+      <c r="D173" s="32" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="174">
-      <c r="C174" s="20" t="s">
+    <row r="174" spans="1:4" ht="13.2">
+      <c r="C174" s="19" t="s">
         <v>352</v>
       </c>
-      <c r="D174" s="33" t="s">
+      <c r="D174" s="32" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="32"/>
-      <c r="B175" s="32" t="s">
+    <row r="175" spans="1:4" ht="13.2">
+      <c r="A175" s="31"/>
+      <c r="B175" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="C175" s="20" t="s">
+      <c r="C175" s="19" t="s">
         <v>355</v>
       </c>
-      <c r="D175" s="33" t="s">
+      <c r="D175" s="32" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="176">
-      <c r="C176" s="20" t="s">
+    <row r="176" spans="1:4" ht="13.2">
+      <c r="C176" s="19" t="s">
         <v>357</v>
       </c>
-      <c r="D176" s="33" t="s">
+      <c r="D176" s="32" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="177">
-      <c r="C177" s="20" t="s">
+    <row r="177" spans="3:4" ht="13.2">
+      <c r="C177" s="19" t="s">
         <v>359</v>
       </c>
-      <c r="D177" s="33" t="s">
+      <c r="D177" s="32" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="178">
-      <c r="C178" s="20" t="s">
+    <row r="178" spans="3:4" ht="13.2">
+      <c r="C178" s="19" t="s">
         <v>361</v>
       </c>
-      <c r="D178" s="33" t="s">
+      <c r="D178" s="32" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="179">
-      <c r="C179" s="20" t="s">
+    <row r="179" spans="3:4" ht="13.2">
+      <c r="C179" s="19" t="s">
         <v>363</v>
       </c>
-      <c r="D179" s="33" t="s">
+      <c r="D179" s="32" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="180">
-      <c r="C180" s="20" t="s">
+    <row r="180" spans="3:4" ht="13.2">
+      <c r="C180" s="19" t="s">
         <v>365</v>
       </c>
-      <c r="D180" s="33" t="s">
+      <c r="D180" s="32" t="s">
         <v>366</v>
       </c>
     </row>
@@ -4070,182 +4074,182 @@
     <mergeCell ref="D61:E61"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C1"/>
-    <hyperlink r:id="rId2" ref="D4"/>
-    <hyperlink r:id="rId3" ref="D5"/>
-    <hyperlink r:id="rId4" ref="D6"/>
-    <hyperlink r:id="rId5" ref="E6"/>
-    <hyperlink r:id="rId6" ref="F6"/>
-    <hyperlink r:id="rId7" ref="D7"/>
-    <hyperlink r:id="rId8" ref="D8"/>
-    <hyperlink r:id="rId9" ref="D9"/>
-    <hyperlink r:id="rId10" ref="D10"/>
-    <hyperlink r:id="rId11" ref="D11"/>
-    <hyperlink r:id="rId12" ref="D12"/>
-    <hyperlink r:id="rId13" ref="D13"/>
-    <hyperlink r:id="rId14" ref="D14"/>
-    <hyperlink r:id="rId15" ref="D15"/>
-    <hyperlink r:id="rId16" ref="E15"/>
-    <hyperlink r:id="rId17" ref="D17"/>
-    <hyperlink r:id="rId18" ref="D18"/>
-    <hyperlink r:id="rId19" ref="D19"/>
-    <hyperlink r:id="rId20" ref="D20"/>
-    <hyperlink r:id="rId21" ref="D21"/>
-    <hyperlink r:id="rId22" ref="D22"/>
-    <hyperlink r:id="rId23" ref="D23"/>
-    <hyperlink r:id="rId24" ref="D24"/>
-    <hyperlink r:id="rId25" ref="D26"/>
-    <hyperlink r:id="rId26" ref="D27"/>
-    <hyperlink r:id="rId27" ref="D28"/>
-    <hyperlink r:id="rId28" ref="D29"/>
-    <hyperlink r:id="rId29" ref="D30"/>
-    <hyperlink r:id="rId30" ref="D31"/>
-    <hyperlink r:id="rId31" ref="D32"/>
-    <hyperlink r:id="rId32" ref="D33"/>
-    <hyperlink r:id="rId33" ref="D34"/>
-    <hyperlink r:id="rId34" ref="D35"/>
-    <hyperlink r:id="rId35" ref="D36"/>
-    <hyperlink r:id="rId36" ref="D37"/>
-    <hyperlink r:id="rId37" ref="D39"/>
-    <hyperlink r:id="rId38" ref="D40"/>
-    <hyperlink r:id="rId39" ref="D41"/>
-    <hyperlink r:id="rId40" ref="D42"/>
-    <hyperlink r:id="rId41" ref="D43"/>
-    <hyperlink r:id="rId42" ref="D44"/>
-    <hyperlink r:id="rId43" ref="D46"/>
-    <hyperlink r:id="rId44" ref="D47"/>
-    <hyperlink r:id="rId45" ref="D48"/>
-    <hyperlink r:id="rId46" ref="D49"/>
-    <hyperlink r:id="rId47" ref="D50"/>
-    <hyperlink r:id="rId48" ref="D51"/>
-    <hyperlink r:id="rId49" ref="D53"/>
-    <hyperlink r:id="rId50" ref="D54"/>
-    <hyperlink r:id="rId51" ref="D55"/>
-    <hyperlink r:id="rId52" ref="D56"/>
-    <hyperlink r:id="rId53" ref="D57"/>
-    <hyperlink r:id="rId54" ref="D58"/>
-    <hyperlink r:id="rId55" ref="D59"/>
-    <hyperlink r:id="rId56" ref="D61"/>
-    <hyperlink r:id="rId57" ref="D62"/>
-    <hyperlink r:id="rId58" ref="D63"/>
-    <hyperlink r:id="rId59" ref="D64"/>
-    <hyperlink r:id="rId60" ref="D65"/>
-    <hyperlink r:id="rId61" ref="D66"/>
-    <hyperlink r:id="rId62" ref="D67"/>
-    <hyperlink r:id="rId63" ref="D68"/>
-    <hyperlink r:id="rId64" ref="D70"/>
-    <hyperlink r:id="rId65" ref="D71"/>
-    <hyperlink r:id="rId66" ref="D72"/>
-    <hyperlink r:id="rId67" ref="D73"/>
-    <hyperlink r:id="rId68" ref="D74"/>
-    <hyperlink r:id="rId69" ref="D75"/>
-    <hyperlink r:id="rId70" ref="C77"/>
-    <hyperlink r:id="rId71" ref="D77"/>
-    <hyperlink r:id="rId72" ref="D78"/>
-    <hyperlink r:id="rId73" ref="D80"/>
-    <hyperlink r:id="rId74" ref="D81"/>
-    <hyperlink r:id="rId75" ref="D82"/>
-    <hyperlink r:id="rId76" ref="D83"/>
-    <hyperlink r:id="rId77" ref="D84"/>
-    <hyperlink r:id="rId78" ref="D85"/>
-    <hyperlink r:id="rId79" ref="D87"/>
-    <hyperlink r:id="rId80" ref="D88"/>
-    <hyperlink r:id="rId81" ref="D89"/>
-    <hyperlink r:id="rId82" ref="D90"/>
-    <hyperlink r:id="rId83" ref="D92"/>
-    <hyperlink r:id="rId84" ref="D93"/>
-    <hyperlink r:id="rId85" ref="D94"/>
-    <hyperlink r:id="rId86" ref="D95"/>
-    <hyperlink r:id="rId87" ref="D96"/>
-    <hyperlink r:id="rId88" ref="D97"/>
-    <hyperlink r:id="rId89" ref="D98"/>
-    <hyperlink r:id="rId90" ref="D99"/>
-    <hyperlink r:id="rId91" ref="D100"/>
-    <hyperlink r:id="rId92" ref="D101"/>
-    <hyperlink r:id="rId93" ref="D102"/>
-    <hyperlink r:id="rId94" ref="D103"/>
-    <hyperlink r:id="rId95" ref="D104"/>
-    <hyperlink r:id="rId96" ref="C105"/>
-    <hyperlink r:id="rId97" ref="D105"/>
-    <hyperlink r:id="rId98" ref="D106"/>
-    <hyperlink r:id="rId99" ref="D107"/>
-    <hyperlink r:id="rId100" ref="D108"/>
-    <hyperlink r:id="rId101" ref="D109"/>
-    <hyperlink r:id="rId102" ref="D110"/>
-    <hyperlink r:id="rId103" ref="D111"/>
-    <hyperlink r:id="rId104" ref="D112"/>
-    <hyperlink r:id="rId105" ref="D113"/>
-    <hyperlink r:id="rId106" ref="D114"/>
-    <hyperlink r:id="rId107" ref="D116"/>
-    <hyperlink r:id="rId108" ref="D117"/>
-    <hyperlink r:id="rId109" ref="D118"/>
-    <hyperlink r:id="rId110" ref="D119"/>
-    <hyperlink r:id="rId111" ref="D120"/>
-    <hyperlink r:id="rId112" ref="D121"/>
-    <hyperlink r:id="rId113" ref="D122"/>
-    <hyperlink r:id="rId114" ref="D123"/>
-    <hyperlink r:id="rId115" ref="D124"/>
-    <hyperlink r:id="rId116" ref="D125"/>
-    <hyperlink r:id="rId117" ref="D126"/>
-    <hyperlink r:id="rId118" ref="D127"/>
-    <hyperlink r:id="rId119" ref="D128"/>
-    <hyperlink r:id="rId120" ref="D129"/>
-    <hyperlink r:id="rId121" ref="D130"/>
-    <hyperlink r:id="rId122" ref="D131"/>
-    <hyperlink r:id="rId123" ref="D132"/>
-    <hyperlink r:id="rId124" ref="D134"/>
-    <hyperlink r:id="rId125" ref="E134"/>
-    <hyperlink r:id="rId126" ref="D135"/>
-    <hyperlink r:id="rId127" ref="E135"/>
-    <hyperlink r:id="rId128" ref="D136"/>
-    <hyperlink r:id="rId129" ref="E136"/>
-    <hyperlink r:id="rId130" ref="D137"/>
-    <hyperlink r:id="rId131" ref="E137"/>
-    <hyperlink r:id="rId132" ref="D138"/>
-    <hyperlink r:id="rId133" ref="E138"/>
-    <hyperlink r:id="rId134" ref="D139"/>
-    <hyperlink r:id="rId135" ref="D140"/>
-    <hyperlink r:id="rId136" ref="E140"/>
-    <hyperlink r:id="rId137" ref="D141"/>
-    <hyperlink r:id="rId138" ref="D142"/>
-    <hyperlink r:id="rId139" ref="D143"/>
-    <hyperlink r:id="rId140" ref="D145"/>
-    <hyperlink r:id="rId141" ref="D146"/>
-    <hyperlink r:id="rId142" ref="D147"/>
-    <hyperlink r:id="rId143" ref="D148"/>
-    <hyperlink r:id="rId144" ref="D149"/>
-    <hyperlink r:id="rId145" ref="D150"/>
-    <hyperlink r:id="rId146" ref="D151"/>
-    <hyperlink r:id="rId147" ref="D152"/>
-    <hyperlink r:id="rId148" ref="D153"/>
-    <hyperlink r:id="rId149" ref="D154"/>
-    <hyperlink r:id="rId150" ref="D155"/>
-    <hyperlink r:id="rId151" ref="D156"/>
-    <hyperlink r:id="rId152" ref="D157"/>
-    <hyperlink r:id="rId153" ref="D158"/>
-    <hyperlink r:id="rId154" ref="D159"/>
-    <hyperlink r:id="rId155" ref="D160"/>
-    <hyperlink r:id="rId156" ref="D161"/>
-    <hyperlink r:id="rId157" ref="D162"/>
-    <hyperlink r:id="rId158" ref="D163"/>
-    <hyperlink r:id="rId159" ref="D164"/>
-    <hyperlink r:id="rId160" ref="D165"/>
-    <hyperlink r:id="rId161" ref="D166"/>
-    <hyperlink r:id="rId162" ref="D167"/>
-    <hyperlink r:id="rId163" ref="D168"/>
-    <hyperlink r:id="rId164" ref="D169"/>
-    <hyperlink r:id="rId165" ref="D170"/>
-    <hyperlink r:id="rId166" ref="D171"/>
-    <hyperlink r:id="rId167" ref="D172"/>
-    <hyperlink r:id="rId168" ref="D173"/>
-    <hyperlink r:id="rId169" ref="D174"/>
-    <hyperlink r:id="rId170" ref="D175"/>
-    <hyperlink r:id="rId171" ref="D176"/>
-    <hyperlink r:id="rId172" ref="D177"/>
-    <hyperlink r:id="rId173" ref="D178"/>
-    <hyperlink r:id="rId174" ref="D179"/>
-    <hyperlink r:id="rId175" ref="D180"/>
+    <hyperlink ref="C1" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F6" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="D7" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="D8" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D9" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D10" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D11" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="D12" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="D13" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="D14" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="D15" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E15" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="D17" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="D18" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="D19" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="D20" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="D21" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="D22" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="D23" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="D24" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="D26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="D27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="D28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="D29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="D30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="D31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="D32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="D33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="D34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="D35" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="D36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="D37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="D39" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="D40" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="D41" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="D42" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="D43" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="D44" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="D46" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="D47" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="D48" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="D49" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="D50" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="D51" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="D53" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="D54" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="D55" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="D56" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="D57" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="D58" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="D59" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="D61" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="D62" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="D63" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="D64" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="D65" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="D66" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="D67" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="D68" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="D70" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="D71" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="D72" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="D73" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="D74" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="D75" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="C77" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="D77" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="D78" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="D80" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="D81" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="D82" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="D83" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="D84" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="D85" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="D87" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="D88" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="D89" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="D90" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="D92" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="D93" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="D94" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="D95" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="D96" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="D97" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="D98" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="D99" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="D100" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="D101" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="D102" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="D103" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="D104" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="C105" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="D105" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="D106" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="D107" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="D108" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="D109" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="D110" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="D111" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="D112" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="D113" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="D114" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="D116" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="D117" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="D118" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="D119" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="D120" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="D121" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="D122" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="D123" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="D124" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="D125" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="D126" r:id="rId117" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="D127" r:id="rId118" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="D128" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="D129" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
+    <hyperlink ref="D130" r:id="rId121" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
+    <hyperlink ref="D131" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
+    <hyperlink ref="D132" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="D134" r:id="rId124" xr:uid="{00000000-0004-0000-0000-00007B000000}"/>
+    <hyperlink ref="E134" r:id="rId125" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
+    <hyperlink ref="D135" r:id="rId126" xr:uid="{00000000-0004-0000-0000-00007D000000}"/>
+    <hyperlink ref="E135" r:id="rId127" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
+    <hyperlink ref="D136" r:id="rId128" xr:uid="{00000000-0004-0000-0000-00007F000000}"/>
+    <hyperlink ref="E136" r:id="rId129" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
+    <hyperlink ref="D137" r:id="rId130" xr:uid="{00000000-0004-0000-0000-000081000000}"/>
+    <hyperlink ref="E137" r:id="rId131" xr:uid="{00000000-0004-0000-0000-000082000000}"/>
+    <hyperlink ref="D138" r:id="rId132" xr:uid="{00000000-0004-0000-0000-000083000000}"/>
+    <hyperlink ref="E138" r:id="rId133" xr:uid="{00000000-0004-0000-0000-000084000000}"/>
+    <hyperlink ref="D139" r:id="rId134" xr:uid="{00000000-0004-0000-0000-000085000000}"/>
+    <hyperlink ref="D140" r:id="rId135" xr:uid="{00000000-0004-0000-0000-000086000000}"/>
+    <hyperlink ref="E140" r:id="rId136" xr:uid="{00000000-0004-0000-0000-000087000000}"/>
+    <hyperlink ref="D141" r:id="rId137" xr:uid="{00000000-0004-0000-0000-000088000000}"/>
+    <hyperlink ref="D142" r:id="rId138" xr:uid="{00000000-0004-0000-0000-000089000000}"/>
+    <hyperlink ref="D143" r:id="rId139" xr:uid="{00000000-0004-0000-0000-00008A000000}"/>
+    <hyperlink ref="D145" r:id="rId140" xr:uid="{00000000-0004-0000-0000-00008B000000}"/>
+    <hyperlink ref="D146" r:id="rId141" xr:uid="{00000000-0004-0000-0000-00008C000000}"/>
+    <hyperlink ref="D147" r:id="rId142" xr:uid="{00000000-0004-0000-0000-00008D000000}"/>
+    <hyperlink ref="D148" r:id="rId143" xr:uid="{00000000-0004-0000-0000-00008E000000}"/>
+    <hyperlink ref="D149" r:id="rId144" xr:uid="{00000000-0004-0000-0000-00008F000000}"/>
+    <hyperlink ref="D150" r:id="rId145" xr:uid="{00000000-0004-0000-0000-000090000000}"/>
+    <hyperlink ref="D151" r:id="rId146" xr:uid="{00000000-0004-0000-0000-000091000000}"/>
+    <hyperlink ref="D152" r:id="rId147" xr:uid="{00000000-0004-0000-0000-000092000000}"/>
+    <hyperlink ref="D153" r:id="rId148" xr:uid="{00000000-0004-0000-0000-000093000000}"/>
+    <hyperlink ref="D154" r:id="rId149" xr:uid="{00000000-0004-0000-0000-000094000000}"/>
+    <hyperlink ref="D155" r:id="rId150" xr:uid="{00000000-0004-0000-0000-000095000000}"/>
+    <hyperlink ref="D156" r:id="rId151" xr:uid="{00000000-0004-0000-0000-000096000000}"/>
+    <hyperlink ref="D157" r:id="rId152" xr:uid="{00000000-0004-0000-0000-000097000000}"/>
+    <hyperlink ref="D158" r:id="rId153" xr:uid="{00000000-0004-0000-0000-000098000000}"/>
+    <hyperlink ref="D159" r:id="rId154" xr:uid="{00000000-0004-0000-0000-000099000000}"/>
+    <hyperlink ref="D160" r:id="rId155" xr:uid="{00000000-0004-0000-0000-00009A000000}"/>
+    <hyperlink ref="D161" r:id="rId156" xr:uid="{00000000-0004-0000-0000-00009B000000}"/>
+    <hyperlink ref="D162" r:id="rId157" xr:uid="{00000000-0004-0000-0000-00009C000000}"/>
+    <hyperlink ref="D163" r:id="rId158" xr:uid="{00000000-0004-0000-0000-00009D000000}"/>
+    <hyperlink ref="D164" r:id="rId159" xr:uid="{00000000-0004-0000-0000-00009E000000}"/>
+    <hyperlink ref="D165" r:id="rId160" xr:uid="{00000000-0004-0000-0000-00009F000000}"/>
+    <hyperlink ref="D166" r:id="rId161" xr:uid="{00000000-0004-0000-0000-0000A0000000}"/>
+    <hyperlink ref="D167" r:id="rId162" xr:uid="{00000000-0004-0000-0000-0000A1000000}"/>
+    <hyperlink ref="D168" r:id="rId163" xr:uid="{00000000-0004-0000-0000-0000A2000000}"/>
+    <hyperlink ref="D169" r:id="rId164" xr:uid="{00000000-0004-0000-0000-0000A3000000}"/>
+    <hyperlink ref="D170" r:id="rId165" xr:uid="{00000000-0004-0000-0000-0000A4000000}"/>
+    <hyperlink ref="D171" r:id="rId166" xr:uid="{00000000-0004-0000-0000-0000A5000000}"/>
+    <hyperlink ref="D172" r:id="rId167" xr:uid="{00000000-0004-0000-0000-0000A6000000}"/>
+    <hyperlink ref="D173" r:id="rId168" xr:uid="{00000000-0004-0000-0000-0000A7000000}"/>
+    <hyperlink ref="D174" r:id="rId169" xr:uid="{00000000-0004-0000-0000-0000A8000000}"/>
+    <hyperlink ref="D175" r:id="rId170" xr:uid="{00000000-0004-0000-0000-0000A9000000}"/>
+    <hyperlink ref="D176" r:id="rId171" xr:uid="{00000000-0004-0000-0000-0000AA000000}"/>
+    <hyperlink ref="D177" r:id="rId172" xr:uid="{00000000-0004-0000-0000-0000AB000000}"/>
+    <hyperlink ref="D178" r:id="rId173" xr:uid="{00000000-0004-0000-0000-0000AC000000}"/>
+    <hyperlink ref="D179" r:id="rId174" xr:uid="{00000000-0004-0000-0000-0000AD000000}"/>
+    <hyperlink ref="D180" r:id="rId175" xr:uid="{00000000-0004-0000-0000-0000AE000000}"/>
   </hyperlinks>
-  <drawing r:id="rId176"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>